<commit_message>
fix(onboarding): PUNTO 5 · préstamos · vuelve al flujo + marca bloque (P4) + plantilla espejo del modal (P1) (#1419)
P4 · alta manual y banner abren el wizard con ?from=empezar · WizardCreatePage (wrapper, no el wizard) vuelve a /empezar/prestamos · syncNucleoFromData marca el bloque prestamos con ≥1 préstamo. P1 · plantilla espejo del modal (columnas opcionales: tipo, demora, 5 comisiones, carencia, destino del capital/deducibilidad, garantía) · retrocompatible con la de 10 · es-ES. Wizard PrestamoPageV2 y Financiación intactos.
</commit_message>
<xml_diff>
--- a/public/templates/plantilla-prestamos-atlas.xlsx
+++ b/public/templates/plantilla-prestamos-atlas.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Atlas" sheetId="1" r:id="rId1"/>
+    <sheet name="Léeme" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -399,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:X2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,6 +433,48 @@
       <c r="J1" t="str">
         <v>Tipo (fijo/variable/mixto)</v>
       </c>
+      <c r="K1" t="str">
+        <v>Tipo de préstamo (hipotecario/personal/linea_credito/otro)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Interés de demora %</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Comisión apertura %</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Comisión mantenimiento €</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Comisión amortización anticipada %</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Comisión modificación condiciones %</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Comisión cancelación total %</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Carencia (ninguna/solo_capital/total)</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Carencia meses</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Destino del capital (adquisicion/reforma/cancelar_deuda/inversion/personal/otra)</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Destino importe €</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Destino %</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Garantía (hipotecaria/personal/pignoraticia)</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Garantía sobre (inmueble alias/RC · informativa)</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -464,10 +507,128 @@
       <c r="J2" t="str">
         <v>fijo</v>
       </c>
+      <c r="K2" t="str">
+        <v>hipotecario</v>
+      </c>
+      <c r="L2">
+        <v>12</v>
+      </c>
+      <c r="M2">
+        <v>0.5</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0.5</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0.5</v>
+      </c>
+      <c r="R2" t="str">
+        <v>ninguna</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2" t="str">
+        <v>adquisicion</v>
+      </c>
+      <c r="U2">
+        <v>80000</v>
+      </c>
+      <c r="V2">
+        <v>100</v>
+      </c>
+      <c r="W2" t="str">
+        <v>hipotecaria</v>
+      </c>
+      <c r="X2" t="str">
+        <v>Piso Centro</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A13"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Plantilla de préstamos · Atlas</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>OBLIGATORIAS · solo "Nombre" y "Principal inicial €". El resto es opcional.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>FECHAS · formato DD/MM/AAAA. IMPORTES · coma decimal (1.234,56).</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>DESTINO DEL CAPITAL · para qué se pidió el dinero (determina la deducibilidad).</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v xml:space="preserve">  · adquisicion/reforma + inmueble vinculado → intereses deducibles en ese inmueble.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v xml:space="preserve">  · una fila admite UN destino. Si un préstamo financia varios inmuebles, créalo</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v xml:space="preserve">    aquí con su destino principal y añade el resto en la ficha del préstamo.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>GARANTÍA · qué responde si no pagas (informativa · NO afecta a la fiscalidad).</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>COMPATIBILIDAD · la plantilla anterior de 10 columnas sigue funcionando.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>